<commit_message>
Delete record: フリー 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -1686,7 +1686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2007,32 +2007,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>36.21</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add record: フリー 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -1686,7 +1686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2007,6 +2007,32 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>33.01</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Edit record: フリー 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -2021,11 +2021,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>33.01</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add record: バッタ 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="バッタ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="バック" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ブレ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="メドレー" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="バック" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ブレ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="バッタ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -468,313 +468,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="15.796875" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="14.8984375" customWidth="1" style="1" min="2" max="8"/>
-    <col width="25.5" customWidth="1" style="1" min="9" max="9"/>
-    <col width="14.8984375" customWidth="1" style="1" min="10" max="14"/>
-    <col width="9.8984375" customWidth="1" style="1" min="15" max="15"/>
-    <col width="14.8984375" customWidth="1" style="1" min="16" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>日付</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>学年</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>距離</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>長水路 or 短水路</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>タイム</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>会場</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(短水路)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(長水路)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="n">
-        <v>45823</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>58.49</v>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "短水路")</f>
-        <v/>
-      </c>
-      <c r="H2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "短水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="I2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "長水路")</f>
-        <v/>
-      </c>
-      <c r="J2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "長水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="n">
-        <v>45956</v>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>52.07</v>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n"/>
-      <c r="M3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>51.12</v>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>53</v>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="M5" s="1" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>49.85</v>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="M6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>53.89</v>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>52.64</v>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="D9:D178" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation sqref="F9:F132 K2:K132" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$N$3:$N$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$M$5:$M$6</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
   <cols>
@@ -1153,7 +846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1457,7 +1150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1680,7 +1373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2036,4 +1729,258 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>学年</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>距離</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>長水路or短水路</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>タイム</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>会場</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>45956</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>52.07</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>53</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>52.64</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add record: バック 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="バック" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ブレ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="バッタ" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="メドレー" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="フリー" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="バッタ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="バック" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -468,390 +468,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="15.796875" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="14.8984375" customWidth="1" style="1" min="2" max="4"/>
-    <col width="14.8984375" customWidth="1" style="12" min="5" max="5"/>
-    <col width="14.8984375" customWidth="1" style="1" min="6" max="8"/>
-    <col width="22" customWidth="1" style="1" min="9" max="9"/>
-    <col width="14.8984375" customWidth="1" style="1" min="10" max="15"/>
-    <col width="9.8984375" customWidth="1" style="1" min="16" max="16"/>
-    <col width="14.8984375" customWidth="1" style="1" min="17" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>日付</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>学年</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>距離</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>長水路 or 短水路</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>タイム</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>会場</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(短水路)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(長水路)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="n">
-        <v>45788</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="n">
-        <v>58.72</v>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "短水路")</f>
-        <v/>
-      </c>
-      <c r="H2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "短水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="I2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "長水路")</f>
-        <v/>
-      </c>
-      <c r="J2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "長水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="n">
-        <v>45815</v>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n"/>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="n">
-        <v>45823</v>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>55.74</v>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="n">
-        <v>45844</v>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>56.07</v>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="n">
-        <v>45942</v>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>52.11</v>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="O6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="n">
-        <v>45956</v>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>49.12</v>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>50.03</v>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>48.34</v>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="n">
-        <v>48.72</v>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="D2:D181" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$O$2:$O$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F181 M2:M181" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$O$5:$O$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K132" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$N$3:$N$3</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
   <cols>
@@ -1150,7 +766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1373,7 +989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1723,6 +1339,260 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>学年</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>距離</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>長水路or短水路</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>タイム</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>会場</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>45956</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>52.07</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>53</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>52.64</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1774,7 +1644,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1790,7 +1660,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.49</v>
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1800,7 +1670,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1812,11 +1682,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52.07</v>
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1826,7 +1696,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1838,11 +1708,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51.12</v>
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1852,7 +1722,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1864,11 +1734,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1878,7 +1748,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1890,11 +1760,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.85</v>
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1904,7 +1774,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1916,11 +1786,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>49.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1930,11 +1800,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46130</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1942,39 +1812,117 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52.64</v>
+        <v>50.03</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
         <v>46152</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>

</xml_diff>

<commit_message>
Add record: メドレー 200m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -7,10 +7,10 @@
   </bookViews>
   <sheets>
     <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="メドレー" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="フリー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="バッタ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="バック" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="フリー" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="バッタ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="バック" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="メドレー" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -772,220 +772,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="15.796875" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="14.8984375" customWidth="1" style="1" min="2" max="4"/>
-    <col width="17" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
-    <col width="14.8984375" customWidth="1" style="1" min="6" max="9"/>
-    <col width="9.8984375" customWidth="1" style="1" min="10" max="10"/>
-    <col width="14.8984375" customWidth="1" style="1" min="11" max="16384"/>
-  </cols>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="17.4" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>学年</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>距離</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>長水路 or 短水路</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>長水路or短水路</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>タイム</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>会場</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="n">
-        <v>45710</v>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>小3</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>4'52"00</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="A2" s="14" t="n">
+        <v>45788</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>50.61</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>45816</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>49.82</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>48.98</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>45844</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>45942</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>44.07</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>45955</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>42.36</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>42.24</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>40.99</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="n">
-        <v>45808</v>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>4'17"24</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="n">
-        <v>45899</v>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>3'50"98</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="n">
-        <v>45991</v>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>3'44"22</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="n">
-        <v>46081</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>3'35"70</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="D2:D181" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$I$2:$I$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$I$5:$I$6</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -995,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1032,7 +1167,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45823</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1048,7 +1183,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50.61</v>
+        <v>58.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1058,7 +1193,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45956</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1070,11 +1205,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>49.82</v>
+        <v>52.07</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1084,7 +1219,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45984</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1096,11 +1231,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>48.98</v>
+        <v>51.12</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1110,7 +1245,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>46033</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1122,11 +1257,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>46.9</v>
+        <v>53</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1136,7 +1271,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46055</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1148,11 +1283,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44.07</v>
+        <v>49.85</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1162,7 +1297,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46075</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1174,11 +1309,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>53.89</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1188,11 +1323,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46130</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1200,25 +1335,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>52.64</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46033</v>
+        <v>46152</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1230,115 +1365,11 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42.36</v>
+        <v>49.1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>42.24</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
           <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1390,7 +1421,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1406,7 +1437,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.49</v>
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1416,7 +1447,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1428,11 +1459,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52.07</v>
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1442,7 +1473,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1454,11 +1485,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51.12</v>
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1468,7 +1499,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1480,11 +1511,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1494,7 +1525,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1506,11 +1537,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.85</v>
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1520,7 +1551,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1532,11 +1563,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>49.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1546,11 +1577,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46130</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1558,41 +1589,119 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52.64</v>
+        <v>50.03</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
         <v>46152</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1644,33 +1753,35 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45788</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>58.72</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'52"00</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1678,25 +1789,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>56.3</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'17"24</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1704,25 +1817,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>55.74</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'50"98</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1730,25 +1845,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>56.07</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'44"22</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1756,33 +1873,35 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>52.11</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'35"70</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45956</v>
+        <v>46172</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1790,141 +1909,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.12</v>
+        <v>207.18</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>50.03</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>48.34</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>48.72</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
           <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>45.85</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add record: ブレ 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ブレ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="バッタ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="バック" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="バッタ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="メドレー" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="バック" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ブレ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -468,301 +468,251 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="15.796875" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="14.8984375" customWidth="1" style="1" min="2" max="8"/>
-    <col width="22.09765625" customWidth="1" style="1" min="9" max="9"/>
-    <col width="14.8984375" customWidth="1" style="1" min="10" max="15"/>
-    <col width="9.8984375" customWidth="1" style="1" min="16" max="16"/>
-    <col width="14.8984375" customWidth="1" style="1" min="17" max="16384"/>
-  </cols>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>学年</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>距離</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>長水路 or 短水路</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>長水路or短水路</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>タイム</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>会場</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(短水路)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>50m ベストタイム(長水路)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>50m 更新日</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n">
-        <v>45788</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>68.26000000000001</v>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "短水路")</f>
-        <v/>
-      </c>
-      <c r="H2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "短水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="I2" s="1">
-        <f>_xlfn.MINIFS(E:E, C:C, 50, D:D, "長水路")</f>
-        <v/>
-      </c>
-      <c r="J2" s="5">
-        <f>INDEX(A:A, MATCH(_xlfn.MINIFS(E:E, D:D, "長水路"), E:E, 0))</f>
-        <v/>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
+      <c r="A2" s="14" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>45956</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>52.07</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>長水路</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="n">
-        <v>45815</v>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="E4" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>53</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>長水路</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
-        <v>66.84</v>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n"/>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="n">
-        <v>45844</v>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>60.52</v>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="n">
-        <v>45955</v>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>56.15</v>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
+      <c r="E7" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>52.64</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>57.26</v>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="O6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>56.39</v>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>54.31</v>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="F2:F8 M2:M5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$O$5:$O$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D180" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$O$2:$O$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K132" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$N$3:$N$3</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -772,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -809,33 +759,35 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45823</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小3</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>58.49</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'52"00</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45956</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -843,25 +795,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>52.07</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'17"24</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45984</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -869,25 +823,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>51.12</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'50"98</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>46033</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -895,25 +851,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>53</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'44"22</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46055</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -921,95 +879,45 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>49.85</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'35"70</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46075</v>
+        <v>46172</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>53.89</v>
+        <v>207.18</v>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>52.64</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="F9" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
@@ -1026,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,35 +971,33 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小3</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'52"00</t>
-        </is>
+      <c r="E2" t="n">
+        <v>58.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45808</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1099,27 +1005,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'17"24</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>56.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45899</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1127,27 +1031,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'50"98</t>
-        </is>
+      <c r="E4" t="n">
+        <v>55.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45991</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1155,27 +1057,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'44"22</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>56.07</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>46081</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1183,47 +1083,201 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'35"70</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>52.11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46172</v>
+        <v>45956</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>49.12</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>50.03</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>小5</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>200</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>207.18</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.85</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,7 +1345,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.72</v>
+        <v>50.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1301,7 +1355,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1317,7 +1371,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>56.3</v>
+        <v>49.82</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1343,7 +1397,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>55.74</v>
+        <v>48.98</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1369,7 +1423,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>56.07</v>
+        <v>46.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1395,7 +1449,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>52.11</v>
+        <v>44.07</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1405,7 +1459,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45956</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1421,7 +1475,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.12</v>
+        <v>43.01</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1447,7 +1501,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>50.03</v>
+        <v>42.75</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1457,7 +1511,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46055</v>
+        <v>46033</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1473,7 +1527,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>48.34</v>
+        <v>42.36</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1483,7 +1537,7 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46075</v>
+        <v>46055</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1495,11 +1549,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>48.9</v>
+        <v>41.5</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1509,11 +1563,11 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>46130</v>
+        <v>46075</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1521,21 +1575,21 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>48.72</v>
+        <v>42.24</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>46152</v>
+        <v>46130</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1551,17 +1605,17 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>45.85</v>
+        <v>40.99</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>46179</v>
+        <v>46152</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1573,13 +1627,39 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>長水路</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>47.75</v>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="E14" t="n">
+        <v>40.89</v>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>
@@ -1596,7 +1676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1649,7 +1729,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50.61</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1659,7 +1739,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>45816</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1675,7 +1755,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>49.82</v>
+        <v>66.84</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1685,7 +1765,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>45823</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1697,11 +1777,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>48.98</v>
+        <v>60.52</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1711,7 +1791,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45844</v>
+        <v>45955</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1723,11 +1803,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>46.9</v>
+        <v>56.15</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1737,7 +1817,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>45942</v>
+        <v>46033</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1749,11 +1829,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44.07</v>
+        <v>57.26</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1763,7 +1843,7 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45955</v>
+        <v>46075</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1775,11 +1855,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>43.01</v>
+        <v>56.39</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1789,11 +1869,11 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45984</v>
+        <v>46130</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1805,21 +1885,21 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42.75</v>
+        <v>54.31</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46033</v>
+        <v>46180</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1827,143 +1907,13 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42.36</v>
+        <v>53.01</v>
       </c>
       <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>46055</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小4</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>42.24</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>40.99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>39.25</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="F14" t="inlineStr">
         <is>
           <t>鈴鹿</t>
         </is>

</xml_diff>

<commit_message>
Delete record: バック 50m
</commit_message>
<xml_diff>
--- a/楓果記録.xlsx
+++ b/楓果記録.xlsx
@@ -1702,7 +1702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2101,32 +2101,6 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>46208</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>47.77</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>